<commit_message>
Streamline instructor schedule workflow
</commit_message>
<xml_diff>
--- a/generated_outputs/Weekly Schedules.xlsx
+++ b/generated_outputs/Weekly Schedules.xlsx
@@ -487,7 +487,11 @@
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Lab 1: Prerequisite may be same-day: M1, LO1: Classify and Analyze Variables (first covered Lecture 2) | Lab 1: Prerequisite may be same-day: M1, LO2: Evaluate Study Design and Its Implications (first covered Lecture 2) | Lab 1: Prerequisite may be same-day: M1, LO3: Use R for Data Management and Exploration (first covered Lecture 2)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -505,7 +509,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Lab 2 (Lecture 4)</t>
+          <t>Lab 2 (Lecture 3)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -515,7 +519,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Lecture 3: Near Labor Day Holiday, Classes Suspended | Lab 2: Near Labor Day Holiday, Classes Suspended</t>
+          <t>Lecture 3: Near Labor Day Holiday, Classes Suspended</t>
         </is>
       </c>
     </row>
@@ -561,7 +565,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>P1-1 (Lecture 8)</t>
+          <t>P1-1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -649,7 +653,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Lecture 16: Near Indigenous People's Day Holiday, Classes Suspended | Lecture 16: Substitute a Monday schedule of classes | Quiz 2: Near Indigenous People's Day Holiday, Classes Suspended | Quiz 2: Near Substitute a Monday schedule of classes | P1-2: Near Indigenous People's Day Holiday, Classes Suspended | P1-2: Near Substitute a Monday schedule of classes</t>
+          <t>Lecture 16: Near Indigenous People's Day Holiday, Classes Suspended | Lecture 16: Substitute a Monday schedule of classes | Quiz 2: Near Indigenous People's Day Holiday, Classes Suspended | Quiz 2: Near Substitute a Monday schedule of classes</t>
         </is>
       </c>
     </row>
@@ -677,7 +681,11 @@
           <t>P2-1: P1 Video</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>P2-1: Prerequisite not yet covered: M3, LO5: Distinguish Statistical vs. Practical Significance (first covered Lecture 28) | P2-1: Prerequisite not yet covered: M4, LO1: Inference for a Difference in Proportions (first covered Lecture 21) | P2-1: Prerequisite not yet covered: M4, LO2: Conduct and Interpret Chi-Square Tests (first covered Lecture 22) | P2-1: Prerequisite not yet covered: M4, LO4: Conduct and Interpret t-Tests (first covered Lecture 24) | P2-1: Prerequisite not yet covered: M4, LO5: Explain Hypothesis Testing and Its Limitations (first covered Lecture 28)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -703,7 +711,11 @@
           <t>Lab 6: Lab6 in-lab activity submission | Tutorial 6 (pre-lab for lab6) | P2 Outline</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Lab 6: Prerequisite not yet covered: M3, LO5: Distinguish Statistical vs. Practical Significance (first covered Lecture 28)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -729,7 +741,11 @@
           <t>P2-2: Lab6 in-lab activity submission</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Quiz 3: Prerequisite not yet covered: M3, LO5: Distinguish Statistical vs. Practical Significance (first covered Lecture 28) | P2-2: Prerequisite not yet covered: M3, LO5: Distinguish Statistical vs. Practical Significance (first covered Lecture 28) | P2-2: Prerequisite not yet covered: M4, LO5: Explain Hypothesis Testing and Its Limitations (first covered Lecture 28)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -755,7 +771,11 @@
           <t>P2-3: P2 Progress Report</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>P2-3: Prerequisite may be same-day: M3, LO5: Distinguish Statistical vs. Practical Significance (first covered Lecture 28) | P2-3: Prerequisite may be same-day: M4, LO5: Explain Hypothesis Testing and Its Limitations (first covered Lecture 28)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -781,7 +801,11 @@
           <t>Lab 7: P2 writeup | Tutorial 7 (pre-lab for lab7)</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Lab 7: Prerequisite may be same-day: M5, LO3: Comparing Bayesian and Frequentist Approaches (first covered Lecture 31)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -809,7 +833,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Lecture 32: Near Thanksgiving Recess | Lab 8: Near Thanksgiving Recess | Lab 8: Classes Resume</t>
+          <t>Lecture 32: Near Thanksgiving Recess | Lab 8: Near Thanksgiving Recess | Lab 8: Classes Resume | Lab 8: Missing prerequisite metadata: add learning-objective tags for Lab 8</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Simplify course schedule inputs
</commit_message>
<xml_diff>
--- a/generated_outputs/Weekly Schedules.xlsx
+++ b/generated_outputs/Weekly Schedules.xlsx
@@ -489,7 +489,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Lab 1: Prerequisite may be same-day: M1, LO1: Classify and Analyze Variables (first covered Lecture 2) | Lab 1: Prerequisite may be same-day: M1, LO2: Evaluate Study Design and Its Implications (first covered Lecture 2) | Lab 1: Prerequisite may be same-day: M1, LO3: Use R for Data Management and Exploration (first covered Lecture 2)</t>
+          <t>Lab 1: Prerequisite may be same-day: M1.L01: Classify and Analyze Variables (first covered Lecture 2) | Lab 1: Prerequisite may be same-day: M1.L02: Evaluate Study Design and Its Implications (first covered Lecture 2) | Lab 1: Prerequisite may be same-day: M1.L03: Use R for Data Management and Exploration (first covered Lecture 2)</t>
         </is>
       </c>
     </row>
@@ -560,17 +560,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Lecture 8: Sampling from a small population, Random Variables (Chapters 3.3–3.4); Quiz 1: tentative; Lecture 9: Continuous Distributions (Chapter 3.5)</t>
+          <t>Lecture 8: Sampling from a small population, Random Variables (Chapters 3.3–3.4); Quiz 1: confirmed; Lecture 9: Continuous Distributions (Chapter 3.5)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>P1-1</t>
+          <t>Project1-1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>P1-1: Lab3 in-lab activity submission</t>
+          <t>Project1-1: Lab3 in-lab activity submission</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -638,17 +638,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Lecture 16: Point estimates and sampling variability, continued (Chapter 5.1); Quiz 2: tentative; Lecture 17: Confidence intervals (Chapter 5.2)</t>
+          <t>Lecture 16: Point estimates and sampling variability, continued (Chapter 5.1); Quiz 2: in the lecture time; Lecture 17: Confidence intervals (Chapter 5.2)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>P1-2</t>
+          <t>Project1-2</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>P1-2: Lab5 in-lab activity submission</t>
+          <t>Project1-2: Lab5 in-lab activity submission</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -673,17 +673,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>P2-1</t>
+          <t>Project2-1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>P2-1: P1 Video</t>
+          <t>Project2-1: Project1 Video</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>P2-1: Prerequisite not yet covered: M3, LO5: Distinguish Statistical vs. Practical Significance (first covered Lecture 28) | P2-1: Prerequisite not yet covered: M4, LO1: Inference for a Difference in Proportions (first covered Lecture 21) | P2-1: Prerequisite not yet covered: M4, LO2: Conduct and Interpret Chi-Square Tests (first covered Lecture 22) | P2-1: Prerequisite not yet covered: M4, LO4: Conduct and Interpret t-Tests (first covered Lecture 24) | P2-1: Prerequisite not yet covered: M4, LO5: Explain Hypothesis Testing and Its Limitations (first covered Lecture 28)</t>
+          <t>Project2-1: Prerequisite not yet covered: M3.L05: Distinguish Statistical vs. Practical Significance (first covered Lecture 28) | Project2-1: Prerequisite not yet covered: M4.L01: Inference for a Difference in Proportions (first covered Lecture 21) | Project2-1: Prerequisite not yet covered: M4.L02: Conduct and Interpret Chi-Square Tests (first covered Lecture 22) | Project2-1: Prerequisite not yet covered: M4.L04: Conduct and Interpret t-Tests (first covered Lecture 24) | Project2-1: Prerequisite not yet covered: M4.L05: Explain Hypothesis Testing and Its Limitations (first covered Lecture 28)</t>
         </is>
       </c>
     </row>
@@ -708,12 +708,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Lab 6: Lab6 in-lab activity submission | Tutorial 6 (pre-lab for lab6) | P2 Outline</t>
+          <t>Lab 6: Lab6 in-lab activity submission | Tutorial 6 (pre-lab for lab6) | Project2 Outline</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Lab 6: Prerequisite not yet covered: M3, LO5: Distinguish Statistical vs. Practical Significance (first covered Lecture 28)</t>
+          <t>Lab 6: Prerequisite not yet covered: M3.L05: Distinguish Statistical vs. Practical Significance (first covered Lecture 28)</t>
         </is>
       </c>
     </row>
@@ -733,17 +733,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>P2-2</t>
+          <t>Project2-2</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>P2-2: Lab6 in-lab activity submission</t>
+          <t>Project2-2: Lab6 in-lab activity submission</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Quiz 3: Prerequisite not yet covered: M3, LO5: Distinguish Statistical vs. Practical Significance (first covered Lecture 28) | P2-2: Prerequisite not yet covered: M3, LO5: Distinguish Statistical vs. Practical Significance (first covered Lecture 28) | P2-2: Prerequisite not yet covered: M4, LO5: Explain Hypothesis Testing and Its Limitations (first covered Lecture 28)</t>
+          <t>Quiz 3: Prerequisite not yet covered: M3.L05: Distinguish Statistical vs. Practical Significance (first covered Lecture 28) | Project2-2: Prerequisite not yet covered: M3.L05: Distinguish Statistical vs. Practical Significance (first covered Lecture 28) | Project2-2: Prerequisite not yet covered: M4.L05: Explain Hypothesis Testing and Its Limitations (first covered Lecture 28)</t>
         </is>
       </c>
     </row>
@@ -763,17 +763,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>P2-3</t>
+          <t>Project2-3</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>P2-3: P2 Progress Report</t>
+          <t>Project2-3: Project2 Progress Report</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>P2-3: Prerequisite may be same-day: M3, LO5: Distinguish Statistical vs. Practical Significance (first covered Lecture 28) | P2-3: Prerequisite may be same-day: M4, LO5: Explain Hypothesis Testing and Its Limitations (first covered Lecture 28)</t>
+          <t>Project2-3: Prerequisite may be same-day: M3.L05: Distinguish Statistical vs. Practical Significance (first covered Lecture 28) | Project2-3: Prerequisite may be same-day: M4.L05: Explain Hypothesis Testing and Its Limitations (first covered Lecture 28)</t>
         </is>
       </c>
     </row>
@@ -798,12 +798,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Lab 7: P2 writeup | Tutorial 7 (pre-lab for lab7)</t>
+          <t>Lab 7: Project2 writeup | Tutorial 7 (pre-lab for lab7)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Lab 7: Prerequisite may be same-day: M5, LO3: Comparing Bayesian and Frequentist Approaches (first covered Lecture 31)</t>
+          <t>Lab 7: Prerequisite may be same-day: M5.L03: Comparing Bayesian and Frequentist Approaches (first covered Lecture 31)</t>
         </is>
       </c>
     </row>
@@ -828,7 +828,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Lab 8: P2 Resubmission</t>
+          <t>Lab 8: Project2 Resubmission</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">

</xml_diff>